<commit_message>
fixed: fit ui size + plot to/from pacman
</commit_message>
<xml_diff>
--- a/gal/Assets/Resources/VNovelizerRes/ExcelVNScripts/序章.xlsx
+++ b/gal/Assets/Resources/VNovelizerRes/ExcelVNScripts/序章.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="12080"/>
+    <workbookView windowWidth="24750" windowHeight="12790"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -135,6 +135,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>扑街之后我忍着痛打电话给了交警，有车给我送到了医院，这边出具的伤情鉴定</t>
     </r>
     <r>
@@ -183,6 +189,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>如此这般，我听出来护士那头不想让我下床了，我这么健康的身体哪用顾虑这么多，</t>
     </r>
     <r>
@@ -216,6 +228,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>我打开手机随便翻看，视线没有聚焦在那些滚动的文字上，本来</t>
     </r>
     <r>
@@ -249,6 +267,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>发型感觉是我学生时代经常见到的蘑菇头，到刚才为止她的视线应该还</t>
     </r>
     <r>
@@ -285,6 +309,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
       <t>沉默</t>
     </r>
     <r>
@@ -330,6 +360,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
       <t>医生叔叔说</t>
     </r>
     <r>
@@ -365,6 +401,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
       <t>他说我有糖尿病</t>
     </r>
     <r>
@@ -379,6 +421,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
       <t>糖尿病</t>
     </r>
     <r>
@@ -402,6 +450,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>在我的软磨硬泡之下，她还是把糖收好了，这位叫做“小妍”的女孩</t>
     </r>
     <r>
@@ -1085,7 +1139,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1109,7 +1163,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="49">
@@ -1536,7 +1589,6 @@
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
-      <c r="K3"/>
       <c r="L3" s="2"/>
     </row>
     <row r="4" spans="1:15">
@@ -2540,7 +2592,6 @@
       <c r="H49" s="2"/>
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
-      <c r="K49"/>
       <c r="L49" s="2"/>
     </row>
     <row r="50" spans="1:12">
@@ -2580,676 +2631,676 @@
       <c r="L51" s="2"/>
     </row>
     <row r="52" spans="1:12">
-      <c r="A52" s="11">
+      <c r="A52" s="2">
         <v>1050</v>
       </c>
-      <c r="B52" s="11"/>
-      <c r="C52" s="11"/>
-      <c r="D52" s="11"/>
-      <c r="E52" s="11"/>
-      <c r="F52" s="11"/>
-      <c r="G52" s="11"/>
-      <c r="H52" s="11"/>
-      <c r="I52" s="11"/>
-      <c r="J52" s="11"/>
-      <c r="K52" s="11"/>
-      <c r="L52" s="11"/>
+      <c r="B52" s="2"/>
+      <c r="C52" s="2"/>
+      <c r="D52" s="2"/>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+      <c r="G52" s="2"/>
+      <c r="H52" s="2"/>
+      <c r="I52" s="2"/>
+      <c r="J52" s="2"/>
+      <c r="K52" s="2"/>
+      <c r="L52" s="2"/>
     </row>
     <row r="53" spans="1:12">
-      <c r="A53" s="11">
+      <c r="A53" s="2">
         <v>1051</v>
       </c>
-      <c r="B53" s="11"/>
-      <c r="C53" s="11"/>
-      <c r="D53" s="11"/>
-      <c r="E53" s="11"/>
-      <c r="F53" s="11"/>
-      <c r="G53" s="11"/>
-      <c r="H53" s="11"/>
-      <c r="I53" s="11"/>
-      <c r="J53" s="11"/>
-      <c r="K53" s="11"/>
-      <c r="L53" s="11"/>
+      <c r="B53" s="2"/>
+      <c r="C53" s="2"/>
+      <c r="D53" s="2"/>
+      <c r="E53" s="2"/>
+      <c r="F53" s="2"/>
+      <c r="G53" s="2"/>
+      <c r="H53" s="2"/>
+      <c r="I53" s="2"/>
+      <c r="J53" s="2"/>
+      <c r="K53" s="2"/>
+      <c r="L53" s="2"/>
     </row>
     <row r="54" spans="1:12">
-      <c r="A54" s="11">
+      <c r="A54" s="2">
         <v>1052</v>
       </c>
-      <c r="B54" s="11"/>
-      <c r="C54" s="11"/>
-      <c r="D54" s="11"/>
-      <c r="E54" s="11"/>
-      <c r="F54" s="11"/>
-      <c r="G54" s="11"/>
-      <c r="H54" s="11"/>
-      <c r="I54" s="11"/>
-      <c r="J54" s="11"/>
-      <c r="K54" s="11"/>
-      <c r="L54" s="11"/>
+      <c r="B54" s="2"/>
+      <c r="C54" s="2"/>
+      <c r="D54" s="2"/>
+      <c r="E54" s="2"/>
+      <c r="F54" s="2"/>
+      <c r="G54" s="2"/>
+      <c r="H54" s="2"/>
+      <c r="I54" s="2"/>
+      <c r="J54" s="2"/>
+      <c r="K54" s="2"/>
+      <c r="L54" s="2"/>
     </row>
     <row r="55" spans="1:12">
-      <c r="A55" s="11">
+      <c r="A55" s="2">
         <v>1053</v>
       </c>
-      <c r="B55" s="11"/>
-      <c r="C55" s="11"/>
-      <c r="D55" s="11"/>
-      <c r="E55" s="11"/>
-      <c r="F55" s="11"/>
-      <c r="G55" s="11"/>
-      <c r="H55" s="11"/>
-      <c r="I55" s="11"/>
-      <c r="J55" s="11"/>
-      <c r="K55" s="11"/>
-      <c r="L55" s="11"/>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+      <c r="G55" s="2"/>
+      <c r="H55" s="2"/>
+      <c r="I55" s="2"/>
+      <c r="J55" s="2"/>
+      <c r="K55" s="2"/>
+      <c r="L55" s="2"/>
     </row>
     <row r="56" spans="1:12">
-      <c r="A56" s="11">
+      <c r="A56" s="2">
         <v>1054</v>
       </c>
-      <c r="B56" s="11"/>
-      <c r="C56" s="11"/>
-      <c r="D56" s="11"/>
-      <c r="E56" s="11"/>
-      <c r="F56" s="11"/>
-      <c r="G56" s="11"/>
-      <c r="H56" s="11"/>
-      <c r="I56" s="11"/>
-      <c r="J56" s="11"/>
-      <c r="K56" s="11"/>
-      <c r="L56" s="11"/>
+      <c r="B56" s="2"/>
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
+      <c r="E56" s="2"/>
+      <c r="F56" s="2"/>
+      <c r="G56" s="2"/>
+      <c r="H56" s="2"/>
+      <c r="I56" s="2"/>
+      <c r="J56" s="2"/>
+      <c r="K56" s="2"/>
+      <c r="L56" s="2"/>
     </row>
     <row r="57" spans="1:12">
-      <c r="A57" s="12">
+      <c r="A57" s="11">
         <v>1055</v>
       </c>
-      <c r="B57" s="12"/>
-      <c r="C57" s="12"/>
-      <c r="D57" s="12"/>
-      <c r="E57" s="12"/>
-      <c r="F57" s="12"/>
-      <c r="G57" s="12"/>
-      <c r="H57" s="12"/>
-      <c r="I57" s="12"/>
-      <c r="J57" s="12"/>
-      <c r="K57" s="12"/>
-      <c r="L57" s="12"/>
+      <c r="B57" s="11"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="11"/>
+      <c r="E57" s="11"/>
+      <c r="F57" s="11"/>
+      <c r="G57" s="11"/>
+      <c r="H57" s="11"/>
+      <c r="I57" s="11"/>
+      <c r="J57" s="11"/>
+      <c r="K57" s="11"/>
+      <c r="L57" s="11"/>
     </row>
     <row r="58" spans="1:12">
-      <c r="A58" s="12">
+      <c r="A58" s="11">
         <v>1056</v>
       </c>
-      <c r="B58" s="12"/>
-      <c r="C58" s="12"/>
-      <c r="D58" s="12"/>
-      <c r="E58" s="12"/>
-      <c r="F58" s="12"/>
-      <c r="G58" s="12"/>
-      <c r="H58" s="12"/>
-      <c r="I58" s="12"/>
-      <c r="J58" s="12"/>
-      <c r="K58" s="12"/>
-      <c r="L58" s="12"/>
+      <c r="B58" s="11"/>
+      <c r="C58" s="11"/>
+      <c r="D58" s="11"/>
+      <c r="E58" s="11"/>
+      <c r="F58" s="11"/>
+      <c r="G58" s="11"/>
+      <c r="H58" s="11"/>
+      <c r="I58" s="11"/>
+      <c r="J58" s="11"/>
+      <c r="K58" s="11"/>
+      <c r="L58" s="11"/>
     </row>
     <row r="59" spans="1:12">
-      <c r="A59" s="12">
+      <c r="A59" s="11">
         <v>1057</v>
       </c>
-      <c r="B59" s="12"/>
-      <c r="C59" s="12"/>
-      <c r="D59" s="12"/>
-      <c r="E59" s="12"/>
-      <c r="F59" s="12"/>
-      <c r="G59" s="12"/>
-      <c r="H59" s="12"/>
-      <c r="I59" s="12"/>
-      <c r="J59" s="12"/>
-      <c r="K59" s="12"/>
-      <c r="L59" s="12"/>
+      <c r="B59" s="11"/>
+      <c r="C59" s="11"/>
+      <c r="D59" s="11"/>
+      <c r="E59" s="11"/>
+      <c r="F59" s="11"/>
+      <c r="G59" s="11"/>
+      <c r="H59" s="11"/>
+      <c r="I59" s="11"/>
+      <c r="J59" s="11"/>
+      <c r="K59" s="11"/>
+      <c r="L59" s="11"/>
     </row>
     <row r="60" spans="1:12">
-      <c r="A60" s="12">
+      <c r="A60" s="11">
         <v>1058</v>
       </c>
-      <c r="B60" s="12"/>
-      <c r="C60" s="12"/>
-      <c r="D60" s="12"/>
-      <c r="E60" s="12"/>
-      <c r="F60" s="12"/>
-      <c r="G60" s="12"/>
-      <c r="H60" s="12"/>
-      <c r="I60" s="12"/>
-      <c r="J60" s="12"/>
-      <c r="K60" s="12"/>
-      <c r="L60" s="12"/>
+      <c r="B60" s="11"/>
+      <c r="C60" s="11"/>
+      <c r="D60" s="11"/>
+      <c r="E60" s="11"/>
+      <c r="F60" s="11"/>
+      <c r="G60" s="11"/>
+      <c r="H60" s="11"/>
+      <c r="I60" s="11"/>
+      <c r="J60" s="11"/>
+      <c r="K60" s="11"/>
+      <c r="L60" s="11"/>
     </row>
     <row r="61" spans="1:12">
-      <c r="A61" s="12">
+      <c r="A61" s="11">
         <v>1059</v>
       </c>
-      <c r="B61" s="12"/>
-      <c r="C61" s="12"/>
-      <c r="D61" s="12"/>
-      <c r="E61" s="12"/>
-      <c r="F61" s="12"/>
-      <c r="G61" s="12"/>
-      <c r="H61" s="12"/>
-      <c r="I61" s="12"/>
-      <c r="J61" s="12"/>
-      <c r="K61" s="12"/>
-      <c r="L61" s="12"/>
+      <c r="B61" s="11"/>
+      <c r="C61" s="11"/>
+      <c r="D61" s="11"/>
+      <c r="E61" s="11"/>
+      <c r="F61" s="11"/>
+      <c r="G61" s="11"/>
+      <c r="H61" s="11"/>
+      <c r="I61" s="11"/>
+      <c r="J61" s="11"/>
+      <c r="K61" s="11"/>
+      <c r="L61" s="11"/>
     </row>
     <row r="62" spans="1:12">
-      <c r="A62" s="12">
+      <c r="A62" s="11">
         <v>1060</v>
       </c>
-      <c r="B62" s="12"/>
-      <c r="C62" s="12"/>
-      <c r="D62" s="12"/>
-      <c r="E62" s="12"/>
-      <c r="F62" s="12"/>
-      <c r="G62" s="12"/>
-      <c r="H62" s="12"/>
-      <c r="I62" s="12"/>
-      <c r="J62" s="12"/>
-      <c r="K62" s="12"/>
-      <c r="L62" s="12"/>
+      <c r="B62" s="11"/>
+      <c r="C62" s="11"/>
+      <c r="D62" s="11"/>
+      <c r="E62" s="11"/>
+      <c r="F62" s="11"/>
+      <c r="G62" s="11"/>
+      <c r="H62" s="11"/>
+      <c r="I62" s="11"/>
+      <c r="J62" s="11"/>
+      <c r="K62" s="11"/>
+      <c r="L62" s="11"/>
     </row>
     <row r="63" spans="1:12">
-      <c r="A63" s="12">
+      <c r="A63" s="11">
         <v>1061</v>
       </c>
-      <c r="B63" s="12"/>
-      <c r="C63" s="12"/>
-      <c r="D63" s="12"/>
-      <c r="E63" s="12"/>
-      <c r="F63" s="12"/>
-      <c r="G63" s="12"/>
-      <c r="H63" s="12"/>
-      <c r="I63" s="12"/>
-      <c r="J63" s="12"/>
-      <c r="K63" s="12"/>
-      <c r="L63" s="12"/>
+      <c r="B63" s="11"/>
+      <c r="C63" s="11"/>
+      <c r="D63" s="11"/>
+      <c r="E63" s="11"/>
+      <c r="F63" s="11"/>
+      <c r="G63" s="11"/>
+      <c r="H63" s="11"/>
+      <c r="I63" s="11"/>
+      <c r="J63" s="11"/>
+      <c r="K63" s="11"/>
+      <c r="L63" s="11"/>
     </row>
     <row r="64" spans="1:12">
-      <c r="A64" s="12">
+      <c r="A64" s="11">
         <v>1062</v>
       </c>
-      <c r="B64" s="12"/>
-      <c r="C64" s="12"/>
-      <c r="D64" s="12"/>
-      <c r="E64" s="12"/>
-      <c r="F64" s="12"/>
-      <c r="G64" s="12"/>
-      <c r="H64" s="12"/>
-      <c r="I64" s="12"/>
-      <c r="J64" s="12"/>
-      <c r="K64" s="12"/>
-      <c r="L64" s="12"/>
+      <c r="B64" s="11"/>
+      <c r="C64" s="11"/>
+      <c r="D64" s="11"/>
+      <c r="E64" s="11"/>
+      <c r="F64" s="11"/>
+      <c r="G64" s="11"/>
+      <c r="H64" s="11"/>
+      <c r="I64" s="11"/>
+      <c r="J64" s="11"/>
+      <c r="K64" s="11"/>
+      <c r="L64" s="11"/>
     </row>
     <row r="65" spans="1:12">
-      <c r="A65" s="12">
+      <c r="A65" s="11">
         <v>1063</v>
       </c>
-      <c r="B65" s="12"/>
-      <c r="C65" s="12"/>
-      <c r="D65" s="12"/>
-      <c r="E65" s="12"/>
-      <c r="F65" s="12"/>
-      <c r="G65" s="12"/>
-      <c r="H65" s="12"/>
-      <c r="I65" s="12"/>
-      <c r="J65" s="12"/>
-      <c r="K65" s="12"/>
-      <c r="L65" s="12"/>
+      <c r="B65" s="11"/>
+      <c r="C65" s="11"/>
+      <c r="D65" s="11"/>
+      <c r="E65" s="11"/>
+      <c r="F65" s="11"/>
+      <c r="G65" s="11"/>
+      <c r="H65" s="11"/>
+      <c r="I65" s="11"/>
+      <c r="J65" s="11"/>
+      <c r="K65" s="11"/>
+      <c r="L65" s="11"/>
     </row>
     <row r="66" spans="1:12">
-      <c r="A66" s="12">
+      <c r="A66" s="11">
         <v>1064</v>
       </c>
-      <c r="B66" s="12"/>
-      <c r="C66" s="12"/>
-      <c r="D66" s="12"/>
-      <c r="E66" s="12"/>
-      <c r="F66" s="12"/>
-      <c r="G66" s="12"/>
-      <c r="H66" s="12"/>
-      <c r="I66" s="12"/>
-      <c r="J66" s="12"/>
-      <c r="K66" s="12"/>
-      <c r="L66" s="12"/>
+      <c r="B66" s="11"/>
+      <c r="C66" s="11"/>
+      <c r="D66" s="11"/>
+      <c r="E66" s="11"/>
+      <c r="F66" s="11"/>
+      <c r="G66" s="11"/>
+      <c r="H66" s="11"/>
+      <c r="I66" s="11"/>
+      <c r="J66" s="11"/>
+      <c r="K66" s="11"/>
+      <c r="L66" s="11"/>
     </row>
     <row r="67" spans="1:12">
-      <c r="A67" s="12">
+      <c r="A67" s="11">
         <v>1065</v>
       </c>
-      <c r="B67" s="12"/>
-      <c r="C67" s="12"/>
-      <c r="D67" s="12"/>
-      <c r="E67" s="12"/>
-      <c r="F67" s="12"/>
-      <c r="G67" s="12"/>
-      <c r="H67" s="12"/>
-      <c r="I67" s="12"/>
-      <c r="J67" s="12"/>
-      <c r="K67" s="12"/>
-      <c r="L67" s="12"/>
+      <c r="B67" s="11"/>
+      <c r="C67" s="11"/>
+      <c r="D67" s="11"/>
+      <c r="E67" s="11"/>
+      <c r="F67" s="11"/>
+      <c r="G67" s="11"/>
+      <c r="H67" s="11"/>
+      <c r="I67" s="11"/>
+      <c r="J67" s="11"/>
+      <c r="K67" s="11"/>
+      <c r="L67" s="11"/>
     </row>
     <row r="68" spans="1:12">
-      <c r="A68" s="12">
+      <c r="A68" s="11">
         <v>1066</v>
       </c>
-      <c r="B68" s="12"/>
-      <c r="C68" s="12"/>
-      <c r="D68" s="12"/>
-      <c r="E68" s="12"/>
-      <c r="F68" s="12"/>
-      <c r="G68" s="12"/>
-      <c r="H68" s="12"/>
-      <c r="I68" s="12"/>
-      <c r="J68" s="12"/>
-      <c r="K68" s="12"/>
-      <c r="L68" s="12"/>
+      <c r="B68" s="11"/>
+      <c r="C68" s="11"/>
+      <c r="D68" s="11"/>
+      <c r="E68" s="11"/>
+      <c r="F68" s="11"/>
+      <c r="G68" s="11"/>
+      <c r="H68" s="11"/>
+      <c r="I68" s="11"/>
+      <c r="J68" s="11"/>
+      <c r="K68" s="11"/>
+      <c r="L68" s="11"/>
     </row>
     <row r="69" spans="1:12">
-      <c r="A69" s="12">
+      <c r="A69" s="11">
         <v>1067</v>
       </c>
-      <c r="B69" s="12"/>
-      <c r="C69" s="12"/>
-      <c r="D69" s="12"/>
-      <c r="E69" s="12"/>
-      <c r="F69" s="12"/>
-      <c r="G69" s="12"/>
-      <c r="H69" s="12"/>
-      <c r="I69" s="12"/>
-      <c r="J69" s="12"/>
-      <c r="K69" s="12"/>
-      <c r="L69" s="12"/>
+      <c r="B69" s="11"/>
+      <c r="C69" s="11"/>
+      <c r="D69" s="11"/>
+      <c r="E69" s="11"/>
+      <c r="F69" s="11"/>
+      <c r="G69" s="11"/>
+      <c r="H69" s="11"/>
+      <c r="I69" s="11"/>
+      <c r="J69" s="11"/>
+      <c r="K69" s="11"/>
+      <c r="L69" s="11"/>
     </row>
     <row r="70" spans="1:12">
-      <c r="A70" s="12">
+      <c r="A70" s="11">
         <v>1068</v>
       </c>
-      <c r="B70" s="12"/>
-      <c r="C70" s="12"/>
-      <c r="D70" s="12"/>
-      <c r="E70" s="12"/>
-      <c r="F70" s="12"/>
-      <c r="G70" s="12"/>
-      <c r="H70" s="12"/>
-      <c r="I70" s="12"/>
-      <c r="J70" s="12"/>
-      <c r="K70" s="12"/>
-      <c r="L70" s="12"/>
+      <c r="B70" s="11"/>
+      <c r="C70" s="11"/>
+      <c r="D70" s="11"/>
+      <c r="E70" s="11"/>
+      <c r="F70" s="11"/>
+      <c r="G70" s="11"/>
+      <c r="H70" s="11"/>
+      <c r="I70" s="11"/>
+      <c r="J70" s="11"/>
+      <c r="K70" s="11"/>
+      <c r="L70" s="11"/>
     </row>
     <row r="71" spans="1:12">
-      <c r="A71" s="12">
+      <c r="A71" s="11">
         <v>1069</v>
       </c>
-      <c r="B71" s="12"/>
-      <c r="C71" s="12"/>
-      <c r="D71" s="12"/>
-      <c r="E71" s="12"/>
-      <c r="F71" s="12"/>
-      <c r="G71" s="12"/>
-      <c r="H71" s="12"/>
-      <c r="I71" s="12"/>
-      <c r="J71" s="12"/>
-      <c r="K71" s="12"/>
-      <c r="L71" s="12"/>
+      <c r="B71" s="11"/>
+      <c r="C71" s="11"/>
+      <c r="D71" s="11"/>
+      <c r="E71" s="11"/>
+      <c r="F71" s="11"/>
+      <c r="G71" s="11"/>
+      <c r="H71" s="11"/>
+      <c r="I71" s="11"/>
+      <c r="J71" s="11"/>
+      <c r="K71" s="11"/>
+      <c r="L71" s="11"/>
     </row>
     <row r="72" spans="1:12">
-      <c r="A72" s="12">
+      <c r="A72" s="11">
         <v>1070</v>
       </c>
-      <c r="B72" s="12"/>
-      <c r="C72" s="12"/>
-      <c r="D72" s="12"/>
-      <c r="E72" s="12"/>
-      <c r="F72" s="12"/>
-      <c r="G72" s="12"/>
-      <c r="H72" s="12"/>
-      <c r="I72" s="12"/>
-      <c r="J72" s="12"/>
-      <c r="K72" s="12"/>
-      <c r="L72" s="12"/>
+      <c r="B72" s="11"/>
+      <c r="C72" s="11"/>
+      <c r="D72" s="11"/>
+      <c r="E72" s="11"/>
+      <c r="F72" s="11"/>
+      <c r="G72" s="11"/>
+      <c r="H72" s="11"/>
+      <c r="I72" s="11"/>
+      <c r="J72" s="11"/>
+      <c r="K72" s="11"/>
+      <c r="L72" s="11"/>
     </row>
     <row r="73" spans="1:12">
-      <c r="A73" s="12">
+      <c r="A73" s="11">
         <v>1071</v>
       </c>
-      <c r="B73" s="12"/>
-      <c r="C73" s="12"/>
-      <c r="D73" s="12"/>
-      <c r="E73" s="12"/>
-      <c r="F73" s="12"/>
-      <c r="G73" s="12"/>
-      <c r="H73" s="12"/>
-      <c r="I73" s="12"/>
-      <c r="J73" s="12"/>
-      <c r="K73" s="12"/>
-      <c r="L73" s="12"/>
+      <c r="B73" s="11"/>
+      <c r="C73" s="11"/>
+      <c r="D73" s="11"/>
+      <c r="E73" s="11"/>
+      <c r="F73" s="11"/>
+      <c r="G73" s="11"/>
+      <c r="H73" s="11"/>
+      <c r="I73" s="11"/>
+      <c r="J73" s="11"/>
+      <c r="K73" s="11"/>
+      <c r="L73" s="11"/>
     </row>
     <row r="74" spans="1:12">
-      <c r="A74" s="12">
+      <c r="A74" s="11">
         <v>1072</v>
       </c>
-      <c r="B74" s="12"/>
-      <c r="C74" s="12"/>
-      <c r="D74" s="12"/>
-      <c r="E74" s="12"/>
-      <c r="F74" s="12"/>
-      <c r="G74" s="12"/>
-      <c r="H74" s="12"/>
-      <c r="I74" s="12"/>
-      <c r="J74" s="12"/>
-      <c r="K74" s="12"/>
-      <c r="L74" s="12"/>
+      <c r="B74" s="11"/>
+      <c r="C74" s="11"/>
+      <c r="D74" s="11"/>
+      <c r="E74" s="11"/>
+      <c r="F74" s="11"/>
+      <c r="G74" s="11"/>
+      <c r="H74" s="11"/>
+      <c r="I74" s="11"/>
+      <c r="J74" s="11"/>
+      <c r="K74" s="11"/>
+      <c r="L74" s="11"/>
     </row>
     <row r="75" spans="1:12">
-      <c r="A75" s="12">
+      <c r="A75" s="11">
         <v>1073</v>
       </c>
-      <c r="B75" s="12"/>
-      <c r="C75" s="12"/>
-      <c r="D75" s="12"/>
-      <c r="E75" s="12"/>
-      <c r="F75" s="12"/>
-      <c r="G75" s="12"/>
-      <c r="H75" s="12"/>
-      <c r="I75" s="12"/>
-      <c r="J75" s="12"/>
-      <c r="K75" s="12"/>
-      <c r="L75" s="12"/>
+      <c r="B75" s="11"/>
+      <c r="C75" s="11"/>
+      <c r="D75" s="11"/>
+      <c r="E75" s="11"/>
+      <c r="F75" s="11"/>
+      <c r="G75" s="11"/>
+      <c r="H75" s="11"/>
+      <c r="I75" s="11"/>
+      <c r="J75" s="11"/>
+      <c r="K75" s="11"/>
+      <c r="L75" s="11"/>
     </row>
     <row r="76" spans="1:12">
-      <c r="A76" s="12">
+      <c r="A76" s="11">
         <v>1074</v>
       </c>
-      <c r="B76" s="12"/>
-      <c r="C76" s="12"/>
-      <c r="D76" s="12"/>
-      <c r="E76" s="12"/>
-      <c r="F76" s="12"/>
-      <c r="G76" s="12"/>
-      <c r="H76" s="12"/>
-      <c r="I76" s="12"/>
-      <c r="J76" s="12"/>
-      <c r="K76" s="12"/>
-      <c r="L76" s="12"/>
+      <c r="B76" s="11"/>
+      <c r="C76" s="11"/>
+      <c r="D76" s="11"/>
+      <c r="E76" s="11"/>
+      <c r="F76" s="11"/>
+      <c r="G76" s="11"/>
+      <c r="H76" s="11"/>
+      <c r="I76" s="11"/>
+      <c r="J76" s="11"/>
+      <c r="K76" s="11"/>
+      <c r="L76" s="11"/>
     </row>
     <row r="77" spans="1:12">
-      <c r="A77" s="12">
+      <c r="A77" s="11">
         <v>1075</v>
       </c>
-      <c r="B77" s="12"/>
-      <c r="C77" s="12"/>
-      <c r="D77" s="12"/>
-      <c r="E77" s="12"/>
-      <c r="F77" s="12"/>
-      <c r="G77" s="12"/>
-      <c r="H77" s="12"/>
-      <c r="I77" s="12"/>
-      <c r="J77" s="12"/>
-      <c r="K77" s="12"/>
-      <c r="L77" s="12"/>
+      <c r="B77" s="11"/>
+      <c r="C77" s="11"/>
+      <c r="D77" s="11"/>
+      <c r="E77" s="11"/>
+      <c r="F77" s="11"/>
+      <c r="G77" s="11"/>
+      <c r="H77" s="11"/>
+      <c r="I77" s="11"/>
+      <c r="J77" s="11"/>
+      <c r="K77" s="11"/>
+      <c r="L77" s="11"/>
     </row>
     <row r="78" spans="1:12">
-      <c r="A78" s="12">
+      <c r="A78" s="11">
         <v>1076</v>
       </c>
-      <c r="B78" s="12"/>
-      <c r="C78" s="12"/>
-      <c r="D78" s="12"/>
-      <c r="E78" s="12"/>
-      <c r="F78" s="12"/>
-      <c r="G78" s="12"/>
-      <c r="H78" s="12"/>
-      <c r="I78" s="12"/>
-      <c r="J78" s="12"/>
-      <c r="K78" s="12"/>
-      <c r="L78" s="12"/>
+      <c r="B78" s="11"/>
+      <c r="C78" s="11"/>
+      <c r="D78" s="11"/>
+      <c r="E78" s="11"/>
+      <c r="F78" s="11"/>
+      <c r="G78" s="11"/>
+      <c r="H78" s="11"/>
+      <c r="I78" s="11"/>
+      <c r="J78" s="11"/>
+      <c r="K78" s="11"/>
+      <c r="L78" s="11"/>
     </row>
     <row r="79" spans="1:12">
-      <c r="A79" s="12">
+      <c r="A79" s="11">
         <v>1077</v>
       </c>
-      <c r="B79" s="12"/>
-      <c r="C79" s="12"/>
-      <c r="D79" s="12"/>
-      <c r="E79" s="12"/>
-      <c r="F79" s="12"/>
-      <c r="G79" s="12"/>
-      <c r="H79" s="12"/>
-      <c r="I79" s="12"/>
-      <c r="J79" s="12"/>
-      <c r="K79" s="12"/>
-      <c r="L79" s="12"/>
+      <c r="B79" s="11"/>
+      <c r="C79" s="11"/>
+      <c r="D79" s="11"/>
+      <c r="E79" s="11"/>
+      <c r="F79" s="11"/>
+      <c r="G79" s="11"/>
+      <c r="H79" s="11"/>
+      <c r="I79" s="11"/>
+      <c r="J79" s="11"/>
+      <c r="K79" s="11"/>
+      <c r="L79" s="11"/>
     </row>
     <row r="80" spans="1:12">
-      <c r="A80" s="12">
+      <c r="A80" s="11">
         <v>1078</v>
       </c>
-      <c r="B80" s="12"/>
-      <c r="C80" s="12"/>
-      <c r="D80" s="12"/>
-      <c r="E80" s="12"/>
-      <c r="F80" s="12"/>
-      <c r="G80" s="12"/>
-      <c r="H80" s="12"/>
-      <c r="I80" s="12"/>
-      <c r="J80" s="12"/>
-      <c r="K80" s="12"/>
-      <c r="L80" s="12"/>
+      <c r="B80" s="11"/>
+      <c r="C80" s="11"/>
+      <c r="D80" s="11"/>
+      <c r="E80" s="11"/>
+      <c r="F80" s="11"/>
+      <c r="G80" s="11"/>
+      <c r="H80" s="11"/>
+      <c r="I80" s="11"/>
+      <c r="J80" s="11"/>
+      <c r="K80" s="11"/>
+      <c r="L80" s="11"/>
     </row>
     <row r="81" spans="1:12">
-      <c r="A81" s="12">
+      <c r="A81" s="11">
         <v>1079</v>
       </c>
-      <c r="B81" s="12"/>
-      <c r="C81" s="12"/>
-      <c r="D81" s="12"/>
-      <c r="E81" s="12"/>
-      <c r="F81" s="12"/>
-      <c r="G81" s="12"/>
-      <c r="H81" s="12"/>
-      <c r="I81" s="12"/>
-      <c r="J81" s="12"/>
-      <c r="K81" s="12"/>
-      <c r="L81" s="12"/>
+      <c r="B81" s="11"/>
+      <c r="C81" s="11"/>
+      <c r="D81" s="11"/>
+      <c r="E81" s="11"/>
+      <c r="F81" s="11"/>
+      <c r="G81" s="11"/>
+      <c r="H81" s="11"/>
+      <c r="I81" s="11"/>
+      <c r="J81" s="11"/>
+      <c r="K81" s="11"/>
+      <c r="L81" s="11"/>
     </row>
     <row r="82" spans="1:12">
-      <c r="A82" s="12">
+      <c r="A82" s="11">
         <v>1080</v>
       </c>
-      <c r="B82" s="12"/>
-      <c r="C82" s="12"/>
-      <c r="D82" s="12"/>
-      <c r="E82" s="12"/>
-      <c r="F82" s="12"/>
-      <c r="G82" s="12"/>
-      <c r="H82" s="12"/>
-      <c r="I82" s="12"/>
-      <c r="J82" s="12"/>
-      <c r="K82" s="12"/>
-      <c r="L82" s="12"/>
+      <c r="B82" s="11"/>
+      <c r="C82" s="11"/>
+      <c r="D82" s="11"/>
+      <c r="E82" s="11"/>
+      <c r="F82" s="11"/>
+      <c r="G82" s="11"/>
+      <c r="H82" s="11"/>
+      <c r="I82" s="11"/>
+      <c r="J82" s="11"/>
+      <c r="K82" s="11"/>
+      <c r="L82" s="11"/>
     </row>
     <row r="83" spans="1:12">
-      <c r="A83" s="12">
+      <c r="A83" s="11">
         <v>1081</v>
       </c>
-      <c r="B83" s="12"/>
-      <c r="C83" s="12"/>
-      <c r="D83" s="12"/>
-      <c r="E83" s="12"/>
-      <c r="F83" s="12"/>
-      <c r="G83" s="12"/>
-      <c r="H83" s="12"/>
-      <c r="I83" s="12"/>
-      <c r="J83" s="12"/>
-      <c r="K83" s="12"/>
-      <c r="L83" s="12"/>
+      <c r="B83" s="11"/>
+      <c r="C83" s="11"/>
+      <c r="D83" s="11"/>
+      <c r="E83" s="11"/>
+      <c r="F83" s="11"/>
+      <c r="G83" s="11"/>
+      <c r="H83" s="11"/>
+      <c r="I83" s="11"/>
+      <c r="J83" s="11"/>
+      <c r="K83" s="11"/>
+      <c r="L83" s="11"/>
     </row>
     <row r="84" spans="1:12">
-      <c r="A84" s="12">
+      <c r="A84" s="11">
         <v>1082</v>
       </c>
-      <c r="B84" s="12"/>
-      <c r="C84" s="12"/>
-      <c r="D84" s="12"/>
-      <c r="E84" s="12"/>
-      <c r="F84" s="12"/>
-      <c r="G84" s="12"/>
-      <c r="H84" s="12"/>
-      <c r="I84" s="12"/>
-      <c r="J84" s="12"/>
-      <c r="K84" s="12"/>
-      <c r="L84" s="12"/>
+      <c r="B84" s="11"/>
+      <c r="C84" s="11"/>
+      <c r="D84" s="11"/>
+      <c r="E84" s="11"/>
+      <c r="F84" s="11"/>
+      <c r="G84" s="11"/>
+      <c r="H84" s="11"/>
+      <c r="I84" s="11"/>
+      <c r="J84" s="11"/>
+      <c r="K84" s="11"/>
+      <c r="L84" s="11"/>
     </row>
     <row r="85" spans="1:12">
-      <c r="A85" s="12">
+      <c r="A85" s="11">
         <v>1083</v>
       </c>
-      <c r="B85" s="12"/>
-      <c r="C85" s="12"/>
-      <c r="D85" s="12"/>
-      <c r="E85" s="12"/>
-      <c r="F85" s="12"/>
-      <c r="G85" s="12"/>
-      <c r="H85" s="12"/>
-      <c r="I85" s="12"/>
-      <c r="J85" s="12"/>
-      <c r="K85" s="12"/>
-      <c r="L85" s="12"/>
+      <c r="B85" s="11"/>
+      <c r="C85" s="11"/>
+      <c r="D85" s="11"/>
+      <c r="E85" s="11"/>
+      <c r="F85" s="11"/>
+      <c r="G85" s="11"/>
+      <c r="H85" s="11"/>
+      <c r="I85" s="11"/>
+      <c r="J85" s="11"/>
+      <c r="K85" s="11"/>
+      <c r="L85" s="11"/>
     </row>
     <row r="86" spans="1:12">
-      <c r="A86" s="12">
+      <c r="A86" s="11">
         <v>1084</v>
       </c>
-      <c r="B86" s="12"/>
-      <c r="C86" s="12"/>
-      <c r="D86" s="12"/>
-      <c r="E86" s="12"/>
-      <c r="F86" s="12"/>
-      <c r="G86" s="12"/>
-      <c r="H86" s="12"/>
-      <c r="I86" s="12"/>
-      <c r="J86" s="12"/>
-      <c r="K86" s="12"/>
-      <c r="L86" s="12"/>
+      <c r="B86" s="11"/>
+      <c r="C86" s="11"/>
+      <c r="D86" s="11"/>
+      <c r="E86" s="11"/>
+      <c r="F86" s="11"/>
+      <c r="G86" s="11"/>
+      <c r="H86" s="11"/>
+      <c r="I86" s="11"/>
+      <c r="J86" s="11"/>
+      <c r="K86" s="11"/>
+      <c r="L86" s="11"/>
     </row>
     <row r="87" spans="1:12">
-      <c r="A87" s="12">
+      <c r="A87" s="11">
         <v>1085</v>
       </c>
-      <c r="B87" s="12"/>
-      <c r="C87" s="12"/>
-      <c r="D87" s="12"/>
-      <c r="E87" s="12"/>
-      <c r="F87" s="12"/>
-      <c r="G87" s="12"/>
-      <c r="H87" s="12"/>
-      <c r="I87" s="12"/>
-      <c r="J87" s="12"/>
-      <c r="K87" s="12"/>
-      <c r="L87" s="12"/>
+      <c r="B87" s="11"/>
+      <c r="C87" s="11"/>
+      <c r="D87" s="11"/>
+      <c r="E87" s="11"/>
+      <c r="F87" s="11"/>
+      <c r="G87" s="11"/>
+      <c r="H87" s="11"/>
+      <c r="I87" s="11"/>
+      <c r="J87" s="11"/>
+      <c r="K87" s="11"/>
+      <c r="L87" s="11"/>
     </row>
     <row r="88" spans="1:12">
-      <c r="A88" s="12">
+      <c r="A88" s="11">
         <v>1086</v>
       </c>
-      <c r="B88" s="12"/>
-      <c r="C88" s="12"/>
-      <c r="D88" s="12"/>
-      <c r="E88" s="12"/>
-      <c r="F88" s="12"/>
-      <c r="G88" s="12"/>
-      <c r="H88" s="12"/>
-      <c r="I88" s="12"/>
-      <c r="J88" s="12"/>
-      <c r="K88" s="12"/>
-      <c r="L88" s="12"/>
+      <c r="B88" s="11"/>
+      <c r="C88" s="11"/>
+      <c r="D88" s="11"/>
+      <c r="E88" s="11"/>
+      <c r="F88" s="11"/>
+      <c r="G88" s="11"/>
+      <c r="H88" s="11"/>
+      <c r="I88" s="11"/>
+      <c r="J88" s="11"/>
+      <c r="K88" s="11"/>
+      <c r="L88" s="11"/>
     </row>
     <row r="89" spans="1:12">
-      <c r="A89" s="12">
+      <c r="A89" s="11">
         <v>1087</v>
       </c>
-      <c r="B89" s="12"/>
-      <c r="C89" s="12"/>
-      <c r="D89" s="12"/>
-      <c r="E89" s="12"/>
-      <c r="F89" s="12"/>
-      <c r="G89" s="12"/>
-      <c r="H89" s="12"/>
-      <c r="I89" s="12"/>
-      <c r="J89" s="12"/>
-      <c r="K89" s="12"/>
-      <c r="L89" s="12"/>
+      <c r="B89" s="11"/>
+      <c r="C89" s="11"/>
+      <c r="D89" s="11"/>
+      <c r="E89" s="11"/>
+      <c r="F89" s="11"/>
+      <c r="G89" s="11"/>
+      <c r="H89" s="11"/>
+      <c r="I89" s="11"/>
+      <c r="J89" s="11"/>
+      <c r="K89" s="11"/>
+      <c r="L89" s="11"/>
     </row>
     <row r="90" spans="1:12">
-      <c r="A90" s="12">
+      <c r="A90" s="11">
         <v>1088</v>
       </c>
-      <c r="B90" s="12"/>
-      <c r="C90" s="12"/>
-      <c r="D90" s="12"/>
-      <c r="E90" s="12"/>
-      <c r="F90" s="12"/>
-      <c r="G90" s="12"/>
-      <c r="H90" s="12"/>
-      <c r="I90" s="12"/>
-      <c r="J90" s="12"/>
-      <c r="K90" s="12"/>
-      <c r="L90" s="12"/>
+      <c r="B90" s="11"/>
+      <c r="C90" s="11"/>
+      <c r="D90" s="11"/>
+      <c r="E90" s="11"/>
+      <c r="F90" s="11"/>
+      <c r="G90" s="11"/>
+      <c r="H90" s="11"/>
+      <c r="I90" s="11"/>
+      <c r="J90" s="11"/>
+      <c r="K90" s="11"/>
+      <c r="L90" s="11"/>
     </row>
     <row r="91" spans="1:12">
-      <c r="A91" s="12">
+      <c r="A91" s="11">
         <v>1089</v>
       </c>
-      <c r="B91" s="12"/>
-      <c r="C91" s="12"/>
-      <c r="D91" s="12"/>
-      <c r="E91" s="12"/>
-      <c r="F91" s="12"/>
-      <c r="G91" s="12"/>
-      <c r="H91" s="12"/>
-      <c r="I91" s="12"/>
-      <c r="J91" s="12"/>
-      <c r="K91" s="12"/>
-      <c r="L91" s="12"/>
+      <c r="B91" s="11"/>
+      <c r="C91" s="11"/>
+      <c r="D91" s="11"/>
+      <c r="E91" s="11"/>
+      <c r="F91" s="11"/>
+      <c r="G91" s="11"/>
+      <c r="H91" s="11"/>
+      <c r="I91" s="11"/>
+      <c r="J91" s="11"/>
+      <c r="K91" s="11"/>
+      <c r="L91" s="11"/>
     </row>
     <row r="92" spans="1:12">
-      <c r="A92" s="12">
+      <c r="A92" s="11">
         <v>1090</v>
       </c>
-      <c r="B92" s="12"/>
-      <c r="C92" s="12"/>
-      <c r="D92" s="12"/>
-      <c r="E92" s="12"/>
-      <c r="F92" s="12"/>
-      <c r="G92" s="12"/>
-      <c r="H92" s="12"/>
-      <c r="I92" s="12"/>
-      <c r="J92" s="12"/>
-      <c r="K92" s="12"/>
-      <c r="L92" s="12"/>
+      <c r="B92" s="11"/>
+      <c r="C92" s="11"/>
+      <c r="D92" s="11"/>
+      <c r="E92" s="11"/>
+      <c r="F92" s="11"/>
+      <c r="G92" s="11"/>
+      <c r="H92" s="11"/>
+      <c r="I92" s="11"/>
+      <c r="J92" s="11"/>
+      <c r="K92" s="11"/>
+      <c r="L92" s="11"/>
     </row>
     <row r="93" spans="1:12">
-      <c r="A93" s="12">
+      <c r="A93" s="11">
         <v>1091</v>
       </c>
-      <c r="B93" s="12"/>
-      <c r="C93" s="12"/>
-      <c r="D93" s="12"/>
-      <c r="E93" s="12"/>
-      <c r="F93" s="12"/>
-      <c r="G93" s="12"/>
-      <c r="H93" s="12"/>
-      <c r="I93" s="12"/>
-      <c r="J93" s="12"/>
-      <c r="K93" s="12"/>
-      <c r="L93" s="12"/>
+      <c r="B93" s="11"/>
+      <c r="C93" s="11"/>
+      <c r="D93" s="11"/>
+      <c r="E93" s="11"/>
+      <c r="F93" s="11"/>
+      <c r="G93" s="11"/>
+      <c r="H93" s="11"/>
+      <c r="I93" s="11"/>
+      <c r="J93" s="11"/>
+      <c r="K93" s="11"/>
+      <c r="L93" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Revert "Merge branch 'main' of https://github.com/1256073/SZU-Final-Project"
This reverts commit 2cd73c79e407b17639c717159601b34d13ff5cf8, reversing
changes made to 8bf8d414f7c57c5f7081a275edd6f8646a7adb6f.
</commit_message>
<xml_diff>
--- a/gal/Assets/Resources/VNovelizerRes/ExcelVNScripts/序章.xlsx
+++ b/gal/Assets/Resources/VNovelizerRes/ExcelVNScripts/序章.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="84">
   <si>
     <t>ID</t>
   </si>
@@ -104,22 +104,13 @@
     <t>刹车</t>
   </si>
   <si>
-    <t>choice(创飞黑影|jump(1006))&amp;choice(下意识躲闪|jump(1009))</t>
-  </si>
-  <si>
-    <t>前面路上还有一些碎石，你摔了个狗啃泥</t>
+    <t>choice(创飞黑影|loadScript(序章1,1000))&amp;choice(下意识躲闪|jump(1006))</t>
+  </si>
+  <si>
+    <t>由于惯性和紧张的作用，你摔了个狗啃泥</t>
   </si>
   <si>
     <t>额啊啊</t>
-  </si>
-  <si>
-    <t>刚刚创飞的东西不见了</t>
-  </si>
-  <si>
-    <t>jump(1012)</t>
-  </si>
-  <si>
-    <t>由于惯性和紧张的作用，你摔了个狗啃泥</t>
   </si>
   <si>
     <t>你定睛一看，发现是只黑猫，它观察了你几秒后便跑开了</t>
@@ -1556,6 +1547,9 @@
       <c r="D8" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="E8" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="F8" s="2" t="s">
         <v>13</v>
       </c>
@@ -1601,17 +1595,27 @@
       <c r="B10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
+      <c r="C10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
-      <c r="K10" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="K10" s="2"/>
       <c r="L10" s="2"/>
     </row>
     <row r="11" spans="1:15">
@@ -1619,34 +1623,26 @@
         <v>1009</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>13</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
       <c r="G11" s="2" t="s">
         <v>30</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2" t="s">
-        <v>27</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" ht="77.5" spans="1:15">
       <c r="A12" s="2">
         <v>1010</v>
       </c>
@@ -1657,18 +1653,16 @@
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
-      <c r="G12" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="G12" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" ht="15.5" spans="1:15">
       <c r="A13" s="2">
         <v>1011</v>
       </c>
@@ -1679,13 +1673,13 @@
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
+      <c r="G13" s="7">
+        <v>0.542361111111111</v>
+      </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
-      <c r="K13" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="K13" s="2"/>
       <c r="L13" s="2"/>
     </row>
     <row r="14" spans="1:15">
@@ -1693,26 +1687,16 @@
         <v>1012</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>13</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
       <c r="G14" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>15</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
@@ -1723,26 +1707,22 @@
         <v>1013</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="I15" s="2" t="s">
         <v>35</v>
       </c>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
     </row>
-    <row r="16" ht="77.5" spans="1:15">
+    <row r="16" spans="1:15">
       <c r="A16" s="2">
         <v>1014</v>
       </c>
@@ -1753,7 +1733,7 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
-      <c r="G16" s="6" t="s">
+      <c r="G16" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H16" s="2"/>
@@ -1762,19 +1742,19 @@
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
     </row>
-    <row r="17" ht="15.5" spans="1:12">
+    <row r="17" spans="1:12">
       <c r="A17" s="2">
         <v>1015</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
-      <c r="G17" s="7">
-        <v>0.542361111111111</v>
+      <c r="G17" s="2" t="s">
+        <v>37</v>
       </c>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
@@ -1787,14 +1767,14 @@
         <v>1016</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
@@ -1807,14 +1787,14 @@
         <v>1017</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
@@ -1827,14 +1807,14 @@
         <v>1018</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
@@ -1846,35 +1826,27 @@
       <c r="A21" s="2">
         <v>1019</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
+      <c r="B21" t="s">
+        <v>39</v>
+      </c>
+      <c r="G21" t="s">
+        <v>36</v>
+      </c>
       <c r="L21" s="2"/>
     </row>
-    <row r="22" spans="1:12">
+    <row r="22" ht="28" spans="1:12">
       <c r="A22" s="2">
         <v>1020</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
-      <c r="G22" s="2" t="s">
-        <v>41</v>
+      <c r="G22" s="8" t="s">
+        <v>42</v>
       </c>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
@@ -1882,59 +1854,53 @@
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
     </row>
-    <row r="23" spans="1:12">
+    <row r="23" ht="28" spans="1:12">
       <c r="A23" s="2">
         <v>1021</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2" t="s">
+      <c r="B23" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
       <c r="L23" s="2"/>
     </row>
     <row r="24" spans="1:12">
       <c r="A24" s="2">
         <v>1022</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2" t="s">
+      <c r="B24" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" t="s">
         <v>44</v>
       </c>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
       <c r="L24" s="2"/>
     </row>
     <row r="25" spans="1:12">
       <c r="A25" s="2">
         <v>1023</v>
       </c>
-      <c r="B25" t="s">
-        <v>42</v>
-      </c>
-      <c r="G25" t="s">
-        <v>39</v>
-      </c>
+      <c r="B25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
       <c r="L25" s="2"/>
     </row>
-    <row r="26" ht="28" spans="1:12">
+    <row r="26" spans="1:12">
       <c r="A26" s="2">
         <v>1024</v>
       </c>
@@ -1945,8 +1911,8 @@
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
-      <c r="G26" s="8" t="s">
-        <v>45</v>
+      <c r="G26" s="2" t="s">
+        <v>47</v>
       </c>
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
@@ -1954,31 +1920,49 @@
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
     </row>
-    <row r="27" ht="28" spans="1:12">
+    <row r="27" ht="56" spans="1:12">
       <c r="A27" s="2">
         <v>1025</v>
       </c>
-      <c r="B27" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27" s="9" t="s">
-        <v>46</v>
-      </c>
+      <c r="B27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+      <c r="K27" s="2"/>
       <c r="L27" s="2"/>
     </row>
     <row r="28" spans="1:12">
       <c r="A28" s="2">
         <v>1026</v>
       </c>
-      <c r="B28" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" t="s">
-        <v>47</v>
-      </c>
+      <c r="B28" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
+      <c r="K28" s="2"/>
       <c r="L28" s="2"/>
     </row>
-    <row r="29" spans="1:12">
+    <row r="29" ht="56" spans="1:12">
       <c r="A29" s="2">
         <v>1027</v>
       </c>
@@ -1987,14 +1971,14 @@
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
+      <c r="E29" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="F29" s="2"/>
-      <c r="G29" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="H29" s="2" t="s">
-        <v>49</v>
-      </c>
+      <c r="G29" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="H29" s="2"/>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
@@ -2004,23 +1988,18 @@
       <c r="A30" s="2">
         <v>1028</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
-      <c r="K30" s="2"/>
+      <c r="B30" t="s">
+        <v>13</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G30" t="s">
+        <v>53</v>
+      </c>
       <c r="L30" s="2"/>
     </row>
-    <row r="31" ht="56" spans="1:12">
+    <row r="31" spans="1:12">
       <c r="A31" s="2">
         <v>1029</v>
       </c>
@@ -2031,8 +2010,8 @@
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
-      <c r="G31" s="8" t="s">
-        <v>51</v>
+      <c r="G31" s="10" t="s">
+        <v>54</v>
       </c>
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
@@ -2045,16 +2024,14 @@
         <v>1030</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
-      <c r="E32" s="2" t="s">
-        <v>52</v>
-      </c>
+      <c r="E32" s="2"/>
       <c r="F32" s="2"/>
-      <c r="G32" s="2" t="s">
-        <v>53</v>
+      <c r="G32" s="10" t="s">
+        <v>56</v>
       </c>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
@@ -2062,21 +2039,21 @@
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
     </row>
-    <row r="33" ht="56" spans="1:12">
+    <row r="33" spans="1:12">
       <c r="A33" s="2">
         <v>1031</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F33" s="2"/>
-      <c r="G33" s="8" t="s">
-        <v>54</v>
+      <c r="G33" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
@@ -2088,22 +2065,29 @@
       <c r="A34" s="2">
         <v>1032</v>
       </c>
-      <c r="B34" t="s">
-        <v>13</v>
-      </c>
+      <c r="B34" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
       <c r="E34" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G34" t="s">
-        <v>56</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="F34" s="2"/>
+      <c r="G34" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
       <c r="L34" s="2"/>
     </row>
-    <row r="35" spans="1:12">
+    <row r="35" ht="14.5" spans="1:12">
       <c r="A35" s="2">
         <v>1033</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C35" s="2"/>
@@ -2111,7 +2095,7 @@
       <c r="E35" s="2"/>
       <c r="F35" s="2"/>
       <c r="G35" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
@@ -2124,18 +2108,20 @@
         <v>1034</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>58</v>
+        <v>13</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
       <c r="G36" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
-      <c r="J36" s="2"/>
+      <c r="J36" s="2" t="s">
+        <v>61</v>
+      </c>
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
     </row>
@@ -2143,22 +2129,12 @@
       <c r="A37" s="2">
         <v>1035</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="H37" s="2"/>
-      <c r="I37" s="2"/>
-      <c r="J37" s="2"/>
-      <c r="K37" s="2"/>
+      <c r="B37" t="s">
+        <v>13</v>
+      </c>
+      <c r="G37" t="s">
+        <v>62</v>
+      </c>
       <c r="L37" s="2"/>
     </row>
     <row r="38" spans="1:12">
@@ -2170,12 +2146,10 @@
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
-      <c r="E38" s="2" t="s">
-        <v>55</v>
-      </c>
+      <c r="E38" s="2"/>
       <c r="F38" s="2"/>
       <c r="G38" s="10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
@@ -2183,46 +2157,35 @@
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
     </row>
-    <row r="39" ht="14.5" spans="1:12">
+    <row r="39" spans="1:12">
       <c r="A39" s="2">
         <v>1037</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B39" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
-      <c r="G39" s="10" t="s">
-        <v>62</v>
+      <c r="G39" t="s">
+        <v>64</v>
       </c>
       <c r="H39" s="2"/>
-      <c r="I39" s="2"/>
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
       <c r="L39" s="2"/>
     </row>
-    <row r="40" spans="1:12">
+    <row r="40" ht="28" spans="1:12">
       <c r="A40" s="2">
         <v>1038</v>
       </c>
-      <c r="B40" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
-      <c r="G40" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="H40" s="2"/>
-      <c r="I40" s="2"/>
-      <c r="J40" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="K40" s="2"/>
+      <c r="B40" t="s">
+        <v>13</v>
+      </c>
+      <c r="G40" s="11" t="s">
+        <v>65</v>
+      </c>
       <c r="L40" s="2"/>
     </row>
     <row r="41" spans="1:12">
@@ -2233,27 +2196,19 @@
         <v>13</v>
       </c>
       <c r="G41" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="42" spans="1:12">
       <c r="A42" s="2">
         <v>1040</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
-      <c r="F42" s="2"/>
-      <c r="G42" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H42" s="2"/>
-      <c r="I42" s="2"/>
-      <c r="J42" s="2"/>
-      <c r="K42" s="2"/>
+      <c r="B42" t="s">
+        <v>13</v>
+      </c>
+      <c r="G42" t="s">
+        <v>67</v>
+      </c>
       <c r="L42" s="2"/>
     </row>
     <row r="43" spans="1:12">
@@ -2261,54 +2216,83 @@
         <v>1041</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
       <c r="F43" s="2"/>
-      <c r="G43" t="s">
-        <v>67</v>
+      <c r="G43" s="10" t="s">
+        <v>68</v>
       </c>
       <c r="H43" s="2"/>
+      <c r="I43" s="2"/>
       <c r="J43" s="2"/>
       <c r="K43" s="2"/>
       <c r="L43" s="2"/>
     </row>
-    <row r="44" ht="28" spans="1:12">
+    <row r="44" spans="1:12">
       <c r="A44" s="2">
         <v>1042</v>
       </c>
-      <c r="B44" t="s">
-        <v>13</v>
-      </c>
-      <c r="G44" s="11" t="s">
-        <v>68</v>
-      </c>
+      <c r="B44" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="H44" s="2"/>
+      <c r="I44" s="2"/>
+      <c r="J44" s="2"/>
+      <c r="K44" s="2"/>
       <c r="L44" s="2"/>
     </row>
     <row r="45" spans="1:12">
       <c r="A45" s="2">
         <v>1043</v>
       </c>
-      <c r="B45" t="s">
-        <v>13</v>
-      </c>
-      <c r="G45" t="s">
-        <v>69</v>
-      </c>
+      <c r="B45" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F45" s="2"/>
+      <c r="G45" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="H45" s="2"/>
+      <c r="I45" s="2"/>
+      <c r="J45" s="2"/>
+      <c r="K45" s="2"/>
       <c r="L45" s="2"/>
     </row>
     <row r="46" spans="1:12">
       <c r="A46" s="2">
         <v>1044</v>
       </c>
-      <c r="B46" t="s">
-        <v>13</v>
-      </c>
-      <c r="G46" t="s">
-        <v>70</v>
-      </c>
+      <c r="B46" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F46" s="2"/>
+      <c r="G46" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="H46" s="2"/>
+      <c r="I46" s="2"/>
+      <c r="J46" s="2"/>
+      <c r="K46" s="2"/>
       <c r="L46" s="2"/>
     </row>
     <row r="47" spans="1:12">
@@ -2316,14 +2300,16 @@
         <v>1045</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>58</v>
+        <v>13</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
+      <c r="E47" s="2" t="s">
+        <v>70</v>
+      </c>
       <c r="F47" s="2"/>
-      <c r="G47" s="10" t="s">
-        <v>71</v>
+      <c r="G47" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="H47" s="2"/>
       <c r="I47" s="2"/>
@@ -2340,10 +2326,12 @@
       </c>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
-      <c r="E48" s="2"/>
+      <c r="E48" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="F48" s="2"/>
-      <c r="G48" s="10" t="s">
-        <v>72</v>
+      <c r="G48" s="2" t="s">
+        <v>73</v>
       </c>
       <c r="H48" s="2"/>
       <c r="I48" s="2"/>
@@ -2351,17 +2339,17 @@
       <c r="K48" s="2"/>
       <c r="L48" s="2"/>
     </row>
-    <row r="49" spans="1:12">
+    <row r="49" ht="14.5" spans="1:12">
       <c r="A49" s="2">
         <v>1047</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
       <c r="F49" s="2"/>
       <c r="G49" s="10" t="s">
@@ -2378,7 +2366,7 @@
         <v>1048</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
@@ -2395,21 +2383,21 @@
       <c r="K50" s="2"/>
       <c r="L50" s="2"/>
     </row>
-    <row r="51" spans="1:12">
+    <row r="51" ht="14.5" spans="1:12">
       <c r="A51" s="2">
         <v>1049</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
       <c r="E51" s="2" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
       <c r="F51" s="2"/>
-      <c r="G51" s="2" t="s">
-        <v>37</v>
+      <c r="G51" s="10" t="s">
+        <v>76</v>
       </c>
       <c r="H51" s="2"/>
       <c r="I51" s="2"/>
@@ -2430,8 +2418,8 @@
         <v>13</v>
       </c>
       <c r="F52" s="2"/>
-      <c r="G52" s="2" t="s">
-        <v>76</v>
+      <c r="G52" s="10" t="s">
+        <v>77</v>
       </c>
       <c r="H52" s="2"/>
       <c r="I52" s="2"/>
@@ -2439,34 +2427,24 @@
       <c r="K52" s="2"/>
       <c r="L52" s="2"/>
     </row>
-    <row r="53" ht="14.5" spans="1:12">
+    <row r="53" spans="1:12">
       <c r="A53" s="2">
         <v>1051</v>
       </c>
-      <c r="B53" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
-      <c r="E53" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="F53" s="2"/>
-      <c r="G53" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="H53" s="2"/>
-      <c r="I53" s="2"/>
-      <c r="J53" s="2"/>
-      <c r="K53" s="2"/>
+      <c r="B53" t="s">
+        <v>13</v>
+      </c>
+      <c r="G53" t="s">
+        <v>78</v>
+      </c>
       <c r="L53" s="2"/>
     </row>
-    <row r="54" spans="1:12">
+    <row r="54" ht="28" spans="1:12">
       <c r="A54" s="2">
         <v>1052</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>58</v>
+        <v>13</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
@@ -2474,8 +2452,8 @@
         <v>13</v>
       </c>
       <c r="F54" s="2"/>
-      <c r="G54" s="10" t="s">
-        <v>78</v>
+      <c r="G54" s="8" t="s">
+        <v>79</v>
       </c>
       <c r="H54" s="2"/>
       <c r="I54" s="2"/>
@@ -2483,63 +2461,50 @@
       <c r="K54" s="2"/>
       <c r="L54" s="2"/>
     </row>
-    <row r="55" ht="14.5" spans="1:12">
+    <row r="55" spans="1:12">
       <c r="A55" s="2">
         <v>1053</v>
       </c>
-      <c r="B55" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C55" s="2"/>
-      <c r="D55" s="2"/>
-      <c r="E55" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="F55" s="2"/>
-      <c r="G55" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="H55" s="2"/>
-      <c r="I55" s="2"/>
-      <c r="J55" s="2"/>
-      <c r="K55" s="2"/>
+      <c r="B55" t="s">
+        <v>13</v>
+      </c>
+      <c r="G55" t="s">
+        <v>80</v>
+      </c>
       <c r="L55" s="2"/>
     </row>
     <row r="56" spans="1:12">
       <c r="A56" s="2">
         <v>1054</v>
       </c>
-      <c r="B56" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
-      <c r="E56" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F56" s="2"/>
-      <c r="G56" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="H56" s="2"/>
-      <c r="I56" s="2"/>
-      <c r="J56" s="2"/>
-      <c r="K56" s="2"/>
+      <c r="B56" t="s">
+        <v>13</v>
+      </c>
+      <c r="G56" t="s">
+        <v>81</v>
+      </c>
       <c r="L56" s="2"/>
     </row>
-    <row r="57" spans="1:12">
+    <row r="57" ht="42" spans="1:12">
       <c r="A57" s="12">
         <v>1055</v>
       </c>
-      <c r="B57" t="s">
-        <v>13</v>
-      </c>
-      <c r="G57" t="s">
-        <v>81</v>
-      </c>
+      <c r="B57" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="H57" s="2"/>
+      <c r="I57" s="2"/>
+      <c r="J57" s="2"/>
       <c r="L57" s="12"/>
     </row>
-    <row r="58" ht="28" spans="1:12">
+    <row r="58" spans="1:12">
       <c r="A58" s="12">
         <v>1056</v>
       </c>
@@ -2548,79 +2513,38 @@
       </c>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
-      <c r="E58" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="E58" s="2"/>
       <c r="F58" s="2"/>
-      <c r="G58" s="8" t="s">
-        <v>82</v>
-      </c>
+      <c r="G58" s="2"/>
       <c r="H58" s="2"/>
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
-      <c r="K58" s="2"/>
+      <c r="K58" s="2" t="s">
+        <v>83</v>
+      </c>
       <c r="L58" s="12"/>
     </row>
     <row r="59" spans="1:12">
       <c r="A59" s="12">
         <v>1057</v>
       </c>
-      <c r="B59" t="s">
-        <v>13</v>
-      </c>
-      <c r="G59" t="s">
-        <v>83</v>
-      </c>
       <c r="L59" s="12"/>
     </row>
     <row r="60" spans="1:12">
       <c r="A60" s="12">
         <v>1058</v>
       </c>
-      <c r="B60" t="s">
-        <v>13</v>
-      </c>
-      <c r="G60" t="s">
-        <v>84</v>
-      </c>
       <c r="L60" s="12"/>
     </row>
-    <row r="61" ht="42" spans="1:12">
+    <row r="61" spans="1:12">
       <c r="A61" s="12">
         <v>1059</v>
       </c>
-      <c r="B61" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C61" s="2"/>
-      <c r="D61" s="2"/>
-      <c r="E61" s="2"/>
-      <c r="F61" s="2"/>
-      <c r="G61" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="H61" s="2"/>
-      <c r="I61" s="2"/>
-      <c r="J61" s="2"/>
       <c r="L61" s="12"/>
     </row>
     <row r="62" spans="1:12">
       <c r="A62" s="12">
         <v>1060</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C62" s="2"/>
-      <c r="D62" s="2"/>
-      <c r="E62" s="2"/>
-      <c r="F62" s="2"/>
-      <c r="G62" s="2"/>
-      <c r="H62" s="2"/>
-      <c r="I62" s="2"/>
-      <c r="J62" s="2"/>
-      <c r="K62" s="2" t="s">
-        <v>86</v>
       </c>
       <c r="L62" s="12"/>
     </row>

</xml_diff>